<commit_message>
feat: add KPI scoring sheet to reports and update related tests
</commit_message>
<xml_diff>
--- a/extension/assets/templates/work_report.xlsx
+++ b/extension/assets/templates/work_report.xlsx
@@ -4,8 +4,11 @@
   <workbookPr/>
   <sheets>
     <sheet name="Báo cáo công việc" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Chấm điểm KPI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Chấm điểm KPI'!$A$1:$J$57</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -278,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -448,6 +451,56 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2701,4 +2754,1257 @@
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J57"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col width="9.380000000000001" customWidth="1" style="66" min="1" max="1"/>
+    <col width="18.75" customWidth="1" style="66" min="2" max="2"/>
+    <col width="19.88" customWidth="1" style="66" min="3" max="3"/>
+    <col width="22.13" customWidth="1" style="66" min="4" max="4"/>
+    <col width="10.13" customWidth="1" style="66" min="5" max="5"/>
+    <col width="12.75" customWidth="1" style="66" min="6" max="7"/>
+    <col width="5.13" customWidth="1" style="66" min="8" max="8"/>
+    <col width="23.75" customWidth="1" style="66" min="9" max="9"/>
+    <col width="12.75" customWidth="1" style="66" min="10" max="27"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>BẢNG KPI ĐÁNH GIÁ HIỆU QUẢ CÔNG VIỆC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <f>"Chu kỳ đánh giá: hàng tháng - "&amp;'Báo cáo công việc'!B2</f>
+        <v/>
+      </c>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Cách chấm điểm: Mỗi tiêu chí có điểm tối đa là 5.</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n"/>
+      <c r="B5" s="15" t="n"/>
+      <c r="C5" s="15" t="n"/>
+      <c r="D5" s="15" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="1" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Mức điểm KPI</t>
+        </is>
+      </c>
+      <c r="B6" s="68" t="n"/>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Đánh giá</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Chế độ thưởng/phạt hằng tháng</t>
+        </is>
+      </c>
+      <c r="E6" s="69" t="n"/>
+      <c r="F6" s="69" t="n"/>
+      <c r="G6" s="68" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>4,5 - 5</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="n"/>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Xuất sắc</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Được xếp loại đánh giá Xuất sắc trong tháng đó.</t>
+        </is>
+      </c>
+      <c r="E7" s="69" t="n"/>
+      <c r="F7" s="69" t="n"/>
+      <c r="G7" s="68" t="n"/>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>4 - 4,49</t>
+        </is>
+      </c>
+      <c r="B8" s="68" t="n"/>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Tốt</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Được xếp loại đánh giá Tốt trong tháng đó.</t>
+        </is>
+      </c>
+      <c r="E8" s="69" t="n"/>
+      <c r="F8" s="69" t="n"/>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>3,5 - 3,99</t>
+        </is>
+      </c>
+      <c r="B9" s="68" t="n"/>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Đạt yêu cầu</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>Không có thưởng phạt.</t>
+        </is>
+      </c>
+      <c r="E9" s="69" t="n"/>
+      <c r="F9" s="69" t="n"/>
+      <c r="G9" s="68" t="n"/>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="1" t="n"/>
+      <c r="J9" s="1" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>2,5 - 3,5</t>
+        </is>
+      </c>
+      <c r="B10" s="68" t="n"/>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Kém</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>Bị cảnh cáo hoặc khiển trách. Có thể xem xét bị chuyển vị trí khác.</t>
+        </is>
+      </c>
+      <c r="E10" s="69" t="n"/>
+      <c r="F10" s="69" t="n"/>
+      <c r="G10" s="68" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>&lt; 2,5</t>
+        </is>
+      </c>
+      <c r="B11" s="68" t="n"/>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>Rất kém</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Bị phạt tài chính (5% lương tháng). Có thể xem xét bị chuyển vị trí khác hoặc bị chấm dứt hợp đồng.</t>
+        </is>
+      </c>
+      <c r="E11" s="69" t="n"/>
+      <c r="F11" s="69" t="n"/>
+      <c r="G11" s="68" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="1" t="n"/>
+      <c r="D12" s="1" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="28" t="n"/>
+      <c r="D13" s="28" t="n"/>
+      <c r="E13" s="28" t="n"/>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
+      <c r="H13" s="28" t="n"/>
+      <c r="I13" s="28" t="n"/>
+      <c r="J13" s="1" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>Tiêu chí</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>Chỉ số đo lường</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>Cách đo lường</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>Trọng số</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>Số liệu thực tế</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>Điểm (0-5)</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>Thang điểm</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="n"/>
+      <c r="J14" s="1" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="72" t="inlineStr">
+        <is>
+          <t>Thái độ 
+(Đúng quy trình làm task)</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Estimate / Tổng số task </t>
+        </is>
+      </c>
+      <c r="D15" s="74" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E15" s="75" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F15" s="76">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M27/100)</f>
+        <v/>
+      </c>
+      <c r="G15" s="75">
+        <f>IF(F15="","",IF(F15&gt;=0.8,1,IF(F15&gt;=0.5,2,IF(F15&gt;=0.3,3,IF(F15&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H15" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="77" t="n"/>
+      <c r="B16" s="77" t="n"/>
+      <c r="C16" s="78" t="n"/>
+      <c r="D16" s="78" t="n"/>
+      <c r="E16" s="78" t="n"/>
+      <c r="F16" s="78" t="n"/>
+      <c r="G16" s="78" t="n"/>
+      <c r="H16" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="77" t="n"/>
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="78" t="n"/>
+      <c r="D17" s="78" t="n"/>
+      <c r="E17" s="78" t="n"/>
+      <c r="F17" s="78" t="n"/>
+      <c r="G17" s="78" t="n"/>
+      <c r="H17" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="77" t="n"/>
+      <c r="B18" s="77" t="n"/>
+      <c r="C18" s="78" t="n"/>
+      <c r="D18" s="78" t="n"/>
+      <c r="E18" s="78" t="n"/>
+      <c r="F18" s="78" t="n"/>
+      <c r="G18" s="78" t="n"/>
+      <c r="H18" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I18" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="79" t="n"/>
+      <c r="B19" s="77" t="n"/>
+      <c r="C19" s="70" t="n"/>
+      <c r="D19" s="70" t="n"/>
+      <c r="E19" s="70" t="n"/>
+      <c r="F19" s="70" t="n"/>
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="77" t="n"/>
+      <c r="C20" s="73" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Start date / Tổng số task</t>
+        </is>
+      </c>
+      <c r="D20" s="74" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E20" s="75" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F20" s="76">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M25/100)</f>
+        <v/>
+      </c>
+      <c r="G20" s="75">
+        <f>IF(F20="","",IF(F20&gt;=0.8,1,IF(F20&gt;=0.5,2,IF(F20&gt;=0.3,3,IF(F20&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H20" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="77" t="n"/>
+      <c r="B21" s="77" t="n"/>
+      <c r="C21" s="78" t="n"/>
+      <c r="D21" s="78" t="n"/>
+      <c r="E21" s="78" t="n"/>
+      <c r="F21" s="78" t="n"/>
+      <c r="G21" s="78" t="n"/>
+      <c r="H21" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="77" t="n"/>
+      <c r="B22" s="77" t="n"/>
+      <c r="C22" s="78" t="n"/>
+      <c r="D22" s="78" t="n"/>
+      <c r="E22" s="78" t="n"/>
+      <c r="F22" s="78" t="n"/>
+      <c r="G22" s="78" t="n"/>
+      <c r="H22" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="77" t="n"/>
+      <c r="B23" s="77" t="n"/>
+      <c r="C23" s="78" t="n"/>
+      <c r="D23" s="78" t="n"/>
+      <c r="E23" s="78" t="n"/>
+      <c r="F23" s="78" t="n"/>
+      <c r="G23" s="78" t="n"/>
+      <c r="H23" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="79" t="n"/>
+      <c r="B24" s="77" t="n"/>
+      <c r="C24" s="70" t="n"/>
+      <c r="D24" s="70" t="n"/>
+      <c r="E24" s="70" t="n"/>
+      <c r="F24" s="70" t="n"/>
+      <c r="G24" s="70" t="n"/>
+      <c r="H24" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="77" t="n"/>
+      <c r="C25" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Due date / Tổng số task </t>
+        </is>
+      </c>
+      <c r="D25" s="74" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E25" s="75" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F25" s="76">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M26/100)</f>
+        <v/>
+      </c>
+      <c r="G25" s="75">
+        <f>IF(F25="","",IF(F25&gt;=0.8,1,IF(F25&gt;=0.5,2,IF(F25&gt;=0.3,3,IF(F25&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H25" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="77" t="n"/>
+      <c r="B26" s="77" t="n"/>
+      <c r="C26" s="78" t="n"/>
+      <c r="D26" s="78" t="n"/>
+      <c r="E26" s="78" t="n"/>
+      <c r="F26" s="78" t="n"/>
+      <c r="G26" s="78" t="n"/>
+      <c r="H26" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="77" t="n"/>
+      <c r="B27" s="77" t="n"/>
+      <c r="C27" s="78" t="n"/>
+      <c r="D27" s="78" t="n"/>
+      <c r="E27" s="78" t="n"/>
+      <c r="F27" s="78" t="n"/>
+      <c r="G27" s="78" t="n"/>
+      <c r="H27" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="77" t="n"/>
+      <c r="B28" s="77" t="n"/>
+      <c r="C28" s="78" t="n"/>
+      <c r="D28" s="78" t="n"/>
+      <c r="E28" s="78" t="n"/>
+      <c r="F28" s="78" t="n"/>
+      <c r="G28" s="78" t="n"/>
+      <c r="H28" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="79" t="n"/>
+      <c r="B29" s="77" t="n"/>
+      <c r="C29" s="70" t="n"/>
+      <c r="D29" s="70" t="n"/>
+      <c r="E29" s="70" t="n"/>
+      <c r="F29" s="70" t="n"/>
+      <c r="G29" s="70" t="n"/>
+      <c r="H29" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" s="77" t="n"/>
+      <c r="C30" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Spent time / Tổng số task </t>
+        </is>
+      </c>
+      <c r="D30" s="74" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E30" s="75" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F30" s="76">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M28/100)</f>
+        <v/>
+      </c>
+      <c r="G30" s="75">
+        <f>IF(F30="","",IF(F30&gt;=0.8,1,IF(F30&gt;=0.5,2,IF(F30&gt;=0.3,3,IF(F30&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H30" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="77" t="n"/>
+      <c r="B31" s="77" t="n"/>
+      <c r="C31" s="78" t="n"/>
+      <c r="D31" s="78" t="n"/>
+      <c r="E31" s="78" t="n"/>
+      <c r="F31" s="78" t="n"/>
+      <c r="G31" s="78" t="n"/>
+      <c r="H31" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="77" t="n"/>
+      <c r="B32" s="77" t="n"/>
+      <c r="C32" s="78" t="n"/>
+      <c r="D32" s="78" t="n"/>
+      <c r="E32" s="78" t="n"/>
+      <c r="F32" s="78" t="n"/>
+      <c r="G32" s="78" t="n"/>
+      <c r="H32" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="77" t="n"/>
+      <c r="B33" s="77" t="n"/>
+      <c r="C33" s="78" t="n"/>
+      <c r="D33" s="78" t="n"/>
+      <c r="E33" s="78" t="n"/>
+      <c r="F33" s="78" t="n"/>
+      <c r="G33" s="78" t="n"/>
+      <c r="H33" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I33" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="79" t="n"/>
+      <c r="B34" s="79" t="n"/>
+      <c r="C34" s="70" t="n"/>
+      <c r="D34" s="70" t="n"/>
+      <c r="E34" s="70" t="n"/>
+      <c r="F34" s="70" t="n"/>
+      <c r="G34" s="70" t="n"/>
+      <c r="H34" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I34" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" s="80" t="inlineStr">
+        <is>
+          <t>Khối lượng</t>
+        </is>
+      </c>
+      <c r="C35" s="73" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time / Tổng thời gian làm việc theo lịch công ty</t>
+        </is>
+      </c>
+      <c r="D35" s="74" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E35" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" s="75">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M36)</f>
+        <v/>
+      </c>
+      <c r="G35" s="75">
+        <f>IF(F35="","",IF(F35&gt;=100,5,IF(F35&gt;=90,4,IF(F35&gt;=80,3,IF(F35&gt;=70,2,1)))))</f>
+        <v/>
+      </c>
+      <c r="H35" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 70%</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="77" t="n"/>
+      <c r="B36" s="77" t="n"/>
+      <c r="C36" s="78" t="n"/>
+      <c r="D36" s="78" t="n"/>
+      <c r="E36" s="78" t="n"/>
+      <c r="F36" s="78" t="n"/>
+      <c r="G36" s="78" t="n"/>
+      <c r="H36" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I36" s="40" t="inlineStr">
+        <is>
+          <t>70% - 79%</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="77" t="n"/>
+      <c r="B37" s="77" t="n"/>
+      <c r="C37" s="78" t="n"/>
+      <c r="D37" s="78" t="n"/>
+      <c r="E37" s="78" t="n"/>
+      <c r="F37" s="78" t="n"/>
+      <c r="G37" s="78" t="n"/>
+      <c r="H37" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" s="40" t="inlineStr">
+        <is>
+          <t>80% - 89%</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="77" t="n"/>
+      <c r="B38" s="77" t="n"/>
+      <c r="C38" s="78" t="n"/>
+      <c r="D38" s="78" t="n"/>
+      <c r="E38" s="78" t="n"/>
+      <c r="F38" s="78" t="n"/>
+      <c r="G38" s="78" t="n"/>
+      <c r="H38" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I38" s="40" t="inlineStr">
+        <is>
+          <t>90% - 99%</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="79" t="n"/>
+      <c r="B39" s="79" t="n"/>
+      <c r="C39" s="70" t="n"/>
+      <c r="D39" s="70" t="n"/>
+      <c r="E39" s="70" t="n"/>
+      <c r="F39" s="70" t="n"/>
+      <c r="G39" s="70" t="n"/>
+      <c r="H39" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" s="40" t="inlineStr">
+        <is>
+          <t>≥ 100%</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t>Chất lượng</t>
+        </is>
+      </c>
+      <c r="C40" s="82" t="inlineStr">
+        <is>
+          <t>Tổng số task trễ hạn / Tổng số task</t>
+        </is>
+      </c>
+      <c r="D40" s="40" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E40" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="83">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M31/100)</f>
+        <v/>
+      </c>
+      <c r="G40" s="81">
+        <f>IF(F40="","",IF(F40&gt;=0.8,1,IF(F40&gt;=0.5,2,IF(F40&gt;=0.3,3,IF(F40&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H40" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="77" t="n"/>
+      <c r="B41" s="77" t="n"/>
+      <c r="C41" s="78" t="n"/>
+      <c r="D41" s="78" t="n"/>
+      <c r="E41" s="78" t="n"/>
+      <c r="F41" s="78" t="n"/>
+      <c r="G41" s="78" t="n"/>
+      <c r="H41" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="77" t="n"/>
+      <c r="B42" s="77" t="n"/>
+      <c r="C42" s="78" t="n"/>
+      <c r="D42" s="78" t="n"/>
+      <c r="E42" s="78" t="n"/>
+      <c r="F42" s="78" t="n"/>
+      <c r="G42" s="78" t="n"/>
+      <c r="H42" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I42" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="77" t="n"/>
+      <c r="B43" s="77" t="n"/>
+      <c r="C43" s="78" t="n"/>
+      <c r="D43" s="78" t="n"/>
+      <c r="E43" s="78" t="n"/>
+      <c r="F43" s="78" t="n"/>
+      <c r="G43" s="78" t="n"/>
+      <c r="H43" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I43" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="79" t="n"/>
+      <c r="B44" s="77" t="n"/>
+      <c r="C44" s="70" t="n"/>
+      <c r="D44" s="70" t="n"/>
+      <c r="E44" s="70" t="n"/>
+      <c r="F44" s="70" t="n"/>
+      <c r="G44" s="70" t="n"/>
+      <c r="H44" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I44" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="71" t="n">
+        <v>7</v>
+      </c>
+      <c r="B45" s="77" t="n"/>
+      <c r="C45" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task có bị reopen / Tổng số task </t>
+        </is>
+      </c>
+      <c r="D45" s="40" t="inlineStr">
+        <is>
+          <t>Dữ liệu từ hệ thống Gitlab</t>
+        </is>
+      </c>
+      <c r="E45" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="83">
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M33/100)</f>
+        <v/>
+      </c>
+      <c r="G45" s="81">
+        <f>IF(F45="","",IF(F45&gt;=0.8,1,IF(F45&gt;=0.5,2,IF(F45&gt;=0.3,3,IF(F45&gt;=0.1,4,5)))))</f>
+        <v/>
+      </c>
+      <c r="H45" s="43" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" s="40" t="inlineStr">
+        <is>
+          <t>≥ 80%</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="77" t="n"/>
+      <c r="B46" s="77" t="n"/>
+      <c r="C46" s="78" t="n"/>
+      <c r="D46" s="78" t="n"/>
+      <c r="E46" s="78" t="n"/>
+      <c r="F46" s="78" t="n"/>
+      <c r="G46" s="78" t="n"/>
+      <c r="H46" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" s="40" t="inlineStr">
+        <is>
+          <t>50% - 79%</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="77" t="n"/>
+      <c r="B47" s="77" t="n"/>
+      <c r="C47" s="78" t="n"/>
+      <c r="D47" s="78" t="n"/>
+      <c r="E47" s="78" t="n"/>
+      <c r="F47" s="78" t="n"/>
+      <c r="G47" s="78" t="n"/>
+      <c r="H47" s="43" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" s="40" t="inlineStr">
+        <is>
+          <t>30% - 49%</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="77" t="n"/>
+      <c r="B48" s="77" t="n"/>
+      <c r="C48" s="78" t="n"/>
+      <c r="D48" s="78" t="n"/>
+      <c r="E48" s="78" t="n"/>
+      <c r="F48" s="78" t="n"/>
+      <c r="G48" s="78" t="n"/>
+      <c r="H48" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="I48" s="40" t="inlineStr">
+        <is>
+          <t>10% - 29%</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="n"/>
+    </row>
+    <row r="49" ht="21" customHeight="1" s="66">
+      <c r="A49" s="79" t="n"/>
+      <c r="B49" s="79" t="n"/>
+      <c r="C49" s="70" t="n"/>
+      <c r="D49" s="70" t="n"/>
+      <c r="E49" s="70" t="n"/>
+      <c r="F49" s="70" t="n"/>
+      <c r="G49" s="70" t="n"/>
+      <c r="H49" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="I49" s="40" t="inlineStr">
+        <is>
+          <t>&lt; 10%</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KPI hiệu quả </t>
+        </is>
+      </c>
+      <c r="B50" s="69" t="n"/>
+      <c r="C50" s="69" t="n"/>
+      <c r="D50" s="69" t="n"/>
+      <c r="E50" s="69" t="n"/>
+      <c r="F50" s="68" t="n"/>
+      <c r="G50" s="60">
+        <f>IF('Báo cáo công việc'!M5=0,"",(E15*G15+E20*G20+E25*G25+E30*G30+E35*G35+E40*G40+E45*G45)/10)</f>
+        <v/>
+      </c>
+      <c r="H50" s="13" t="n"/>
+      <c r="I50" s="13" t="n"/>
+      <c r="J50" s="1" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n"/>
+      <c r="B51" s="1" t="n"/>
+      <c r="C51" s="1" t="n"/>
+      <c r="D51" s="1" t="n"/>
+      <c r="E51" s="1" t="n"/>
+      <c r="F51" s="1" t="n"/>
+      <c r="G51" s="1" t="n"/>
+      <c r="H51" s="1" t="n"/>
+      <c r="I51" s="1" t="n"/>
+      <c r="J51" s="1" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="84" t="inlineStr">
+        <is>
+          <t>GIẢI TRÌNH
+(Trình bày các nguyên nhân ảnh hưởng đến các thông số trên - nếu có)</t>
+        </is>
+      </c>
+      <c r="B52" s="69" t="n"/>
+      <c r="C52" s="69" t="n"/>
+      <c r="D52" s="69" t="n"/>
+      <c r="E52" s="69" t="n"/>
+      <c r="F52" s="69" t="n"/>
+      <c r="G52" s="69" t="n"/>
+      <c r="H52" s="69" t="n"/>
+      <c r="I52" s="68" t="n"/>
+      <c r="J52" s="1" t="n"/>
+    </row>
+    <row r="53" ht="48" customHeight="1" s="66">
+      <c r="A53" s="85" t="n"/>
+      <c r="B53" s="69" t="n"/>
+      <c r="C53" s="69" t="n"/>
+      <c r="D53" s="69" t="n"/>
+      <c r="E53" s="69" t="n"/>
+      <c r="F53" s="69" t="n"/>
+      <c r="G53" s="69" t="n"/>
+      <c r="H53" s="69" t="n"/>
+      <c r="I53" s="68" t="n"/>
+      <c r="J53" s="1" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="86" t="inlineStr">
+        <is>
+          <t>TỰ ĐÁNH GIÁ HIỆU QUẢ</t>
+        </is>
+      </c>
+      <c r="B54" s="69" t="n"/>
+      <c r="C54" s="69" t="n"/>
+      <c r="D54" s="69" t="n"/>
+      <c r="E54" s="69" t="n"/>
+      <c r="F54" s="69" t="n"/>
+      <c r="G54" s="69" t="n"/>
+      <c r="H54" s="69" t="n"/>
+      <c r="I54" s="68" t="n"/>
+      <c r="J54" s="1" t="n"/>
+    </row>
+    <row r="55" ht="44.25" customHeight="1" s="66">
+      <c r="A55" s="87" t="n"/>
+      <c r="B55" s="69" t="n"/>
+      <c r="C55" s="69" t="n"/>
+      <c r="D55" s="69" t="n"/>
+      <c r="E55" s="69" t="n"/>
+      <c r="F55" s="69" t="n"/>
+      <c r="G55" s="69" t="n"/>
+      <c r="H55" s="69" t="n"/>
+      <c r="I55" s="68" t="n"/>
+      <c r="J55" s="1" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="86" t="inlineStr">
+        <is>
+          <t>TỰ ĐÁNH GIÁ ĐIỂM CẦN CẢI THIỆN</t>
+        </is>
+      </c>
+      <c r="B56" s="69" t="n"/>
+      <c r="C56" s="69" t="n"/>
+      <c r="D56" s="69" t="n"/>
+      <c r="E56" s="69" t="n"/>
+      <c r="F56" s="69" t="n"/>
+      <c r="G56" s="69" t="n"/>
+      <c r="H56" s="69" t="n"/>
+      <c r="I56" s="68" t="n"/>
+      <c r="J56" s="1" t="n"/>
+    </row>
+    <row r="57" ht="54.75" customHeight="1" s="66">
+      <c r="A57" s="88" t="n"/>
+      <c r="B57" s="69" t="n"/>
+      <c r="C57" s="69" t="n"/>
+      <c r="D57" s="69" t="n"/>
+      <c r="E57" s="69" t="n"/>
+      <c r="F57" s="69" t="n"/>
+      <c r="G57" s="69" t="n"/>
+      <c r="H57" s="69" t="n"/>
+      <c r="I57" s="68" t="n"/>
+      <c r="J57" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="66">
+    <mergeCell ref="C40:C44"/>
+    <mergeCell ref="F35:F39"/>
+    <mergeCell ref="B40:B49"/>
+    <mergeCell ref="E40:E44"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="E30:E34"/>
+    <mergeCell ref="G30:G34"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="E15:E19"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="A20:A24"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A55:I55"/>
+    <mergeCell ref="D15:D19"/>
+    <mergeCell ref="E45:E49"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="G45:G49"/>
+    <mergeCell ref="G35:G39"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="G20:G24"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="A35:A39"/>
+    <mergeCell ref="D25:D29"/>
+    <mergeCell ref="E25:E29"/>
+    <mergeCell ref="G25:G29"/>
+    <mergeCell ref="D20:D24"/>
+    <mergeCell ref="B15:B34"/>
+    <mergeCell ref="A53:I53"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="G40:G44"/>
+    <mergeCell ref="C15:C19"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="D35:D39"/>
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A30:A34"/>
+    <mergeCell ref="C30:C34"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="F25:F29"/>
+    <mergeCell ref="E20:E24"/>
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="A45:A49"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="F15:F19"/>
+    <mergeCell ref="C45:C49"/>
+    <mergeCell ref="F20:F24"/>
+    <mergeCell ref="D40:D44"/>
+    <mergeCell ref="C35:C39"/>
+    <mergeCell ref="F40:F44"/>
+    <mergeCell ref="E35:E39"/>
+    <mergeCell ref="D45:D49"/>
+    <mergeCell ref="F30:F34"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="C20:C24"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C25:C29"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="F45:F49"/>
+    <mergeCell ref="G15:G19"/>
+    <mergeCell ref="A54:I54"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: refactor Excel report generation to JavaScript implementation, update scoring sheet to summarize leave by reason
</commit_message>
<xml_diff>
--- a/extension/assets/templates/work_report.xlsx
+++ b/extension/assets/templates/work_report.xlsx
@@ -885,13 +885,6 @@
       <c r="I4" s="50" t="n"/>
       <c r="J4" s="50" t="n"/>
       <c r="K4" s="1" t="n"/>
-      <c r="L4" s="67" t="inlineStr">
-        <is>
-          <t>Thống Kê</t>
-        </is>
-      </c>
-      <c r="M4" s="68" t="n"/>
-      <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="n"/>
       <c r="P4" s="1" t="n"/>
       <c r="Q4" s="1" t="n"/>
@@ -904,6 +897,13 @@
       <c r="X4" s="1" t="n"/>
       <c r="Y4" s="1" t="n"/>
       <c r="Z4" s="1" t="n"/>
+      <c r="L4" s="67" t="inlineStr">
+        <is>
+          <t>Thống Kê</t>
+        </is>
+      </c>
+      <c r="M4" s="68" t="n"/>
+      <c r="N4" s="1" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="66">
       <c r="A5" s="1" t="n"/>
@@ -953,13 +953,6 @@
         </is>
       </c>
       <c r="K5" s="12" t="n"/>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task </t>
-        </is>
-      </c>
-      <c r="M5" s="25" t="n"/>
-      <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="n"/>
       <c r="P5" s="1" t="n"/>
       <c r="Q5" s="1" t="n"/>
@@ -972,6 +965,13 @@
       <c r="X5" s="1" t="n"/>
       <c r="Y5" s="1" t="n"/>
       <c r="Z5" s="1" t="n"/>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task </t>
+        </is>
+      </c>
+      <c r="M5" s="25" t="n"/>
+      <c r="N5" s="1" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="66">
       <c r="A6" s="1" t="n"/>
@@ -985,13 +985,6 @@
       <c r="I6" s="24" t="n"/>
       <c r="J6" s="24" t="n"/>
       <c r="K6" s="1" t="n"/>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task kế hoạch </t>
-        </is>
-      </c>
-      <c r="M6" s="25" t="n"/>
-      <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
       <c r="P6" s="1" t="n"/>
       <c r="Q6" s="1" t="n"/>
@@ -1004,17 +997,17 @@
       <c r="X6" s="1" t="n"/>
       <c r="Y6" s="1" t="n"/>
       <c r="Z6" s="1" t="n"/>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task kế hoạch </t>
+        </is>
+      </c>
+      <c r="M6" s="25" t="n"/>
+      <c r="N6" s="1" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="66">
       <c r="A7" s="1" t="n"/>
       <c r="K7" s="1" t="n"/>
-      <c r="L7" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task phát sinh </t>
-        </is>
-      </c>
-      <c r="M7" s="25" t="n"/>
-      <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
       <c r="P7" s="1" t="n"/>
       <c r="Q7" s="1" t="n"/>
@@ -1027,23 +1020,17 @@
       <c r="X7" s="1" t="n"/>
       <c r="Y7" s="1" t="n"/>
       <c r="Z7" s="1" t="n"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task phát sinh </t>
+        </is>
+      </c>
+      <c r="M7" s="25" t="n"/>
+      <c r="N7" s="1" t="n"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="66">
       <c r="A8" s="1" t="n"/>
       <c r="K8" s="1" t="n"/>
-      <c r="L8" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian làm việc theo lịch công ty (h)</t>
-        </is>
-      </c>
-      <c r="M8" s="25" t="n">
-        <v>192</v>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Chỗ này luôn để là 192h</t>
-        </is>
-      </c>
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="n"/>
       <c r="Q8" s="1" t="n"/>
@@ -1056,17 +1043,23 @@
       <c r="X8" s="1" t="n"/>
       <c r="Y8" s="1" t="n"/>
       <c r="Z8" s="1" t="n"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian làm việc theo lịch công ty (h)</t>
+        </is>
+      </c>
+      <c r="M8" s="25" t="n">
+        <v>192</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Chỗ này luôn để là 192h</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="66">
       <c r="A9" s="1" t="n"/>
       <c r="K9" s="1" t="n"/>
-      <c r="L9" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Estimate (h)</t>
-        </is>
-      </c>
-      <c r="M9" s="25" t="n"/>
-      <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
       <c r="P9" s="1" t="n"/>
       <c r="Q9" s="1" t="n"/>
@@ -1079,17 +1072,17 @@
       <c r="X9" s="1" t="n"/>
       <c r="Y9" s="1" t="n"/>
       <c r="Z9" s="1" t="n"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Estimate (h)</t>
+        </is>
+      </c>
+      <c r="M9" s="25" t="n"/>
+      <c r="N9" s="1" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="66">
       <c r="A10" s="1" t="n"/>
       <c r="K10" s="1" t="n"/>
-      <c r="L10" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time (h)</t>
-        </is>
-      </c>
-      <c r="M10" s="25" t="n"/>
-      <c r="N10" s="1" t="n"/>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
       <c r="Q10" s="1" t="n"/>
@@ -1102,17 +1095,17 @@
       <c r="X10" s="1" t="n"/>
       <c r="Y10" s="1" t="n"/>
       <c r="Z10" s="1" t="n"/>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time (h)</t>
+        </is>
+      </c>
+      <c r="M10" s="25" t="n"/>
+      <c r="N10" s="1" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="66">
       <c r="A11" s="1" t="n"/>
       <c r="K11" s="1" t="n"/>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time (h) của task kế hoạch </t>
-        </is>
-      </c>
-      <c r="M11" s="25" t="n"/>
-      <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
       <c r="Q11" s="1" t="n"/>
@@ -1125,17 +1118,17 @@
       <c r="X11" s="1" t="n"/>
       <c r="Y11" s="1" t="n"/>
       <c r="Z11" s="1" t="n"/>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time (h) của task kế hoạch </t>
+        </is>
+      </c>
+      <c r="M11" s="25" t="n"/>
+      <c r="N11" s="1" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="66">
       <c r="A12" s="1" t="n"/>
       <c r="K12" s="1" t="n"/>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time (h) của task phát sinh </t>
-        </is>
-      </c>
-      <c r="M12" s="25" t="n"/>
-      <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="n"/>
       <c r="Q12" s="1" t="n"/>
@@ -1148,17 +1141,17 @@
       <c r="X12" s="1" t="n"/>
       <c r="Y12" s="1" t="n"/>
       <c r="Z12" s="1" t="n"/>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time (h) của task phát sinh </t>
+        </is>
+      </c>
+      <c r="M12" s="25" t="n"/>
+      <c r="N12" s="1" t="n"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="66">
       <c r="A13" s="1" t="n"/>
       <c r="K13" s="1" t="n"/>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Start date</t>
-        </is>
-      </c>
-      <c r="M13" s="25" t="n"/>
-      <c r="N13" s="1" t="n"/>
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="n"/>
       <c r="Q13" s="1" t="n"/>
@@ -1171,17 +1164,17 @@
       <c r="X13" s="1" t="n"/>
       <c r="Y13" s="1" t="n"/>
       <c r="Z13" s="1" t="n"/>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Start date</t>
+        </is>
+      </c>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="1" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="66">
       <c r="A14" s="1" t="n"/>
       <c r="K14" s="1" t="n"/>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Due date</t>
-        </is>
-      </c>
-      <c r="M14" s="25" t="n"/>
-      <c r="N14" s="1" t="n"/>
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
       <c r="Q14" s="1" t="n"/>
@@ -1194,17 +1187,17 @@
       <c r="X14" s="1" t="n"/>
       <c r="Y14" s="1" t="n"/>
       <c r="Z14" s="1" t="n"/>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Due date</t>
+        </is>
+      </c>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="1" t="n"/>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="66">
       <c r="A15" s="1" t="n"/>
       <c r="K15" s="1" t="n"/>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Estimate </t>
-        </is>
-      </c>
-      <c r="M15" s="25" t="n"/>
-      <c r="N15" s="1" t="n"/>
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="n"/>
       <c r="Q15" s="1" t="n"/>
@@ -1217,17 +1210,17 @@
       <c r="X15" s="1" t="n"/>
       <c r="Y15" s="1" t="n"/>
       <c r="Z15" s="1" t="n"/>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Estimate </t>
+        </is>
+      </c>
+      <c r="M15" s="25" t="n"/>
+      <c r="N15" s="1" t="n"/>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="66">
       <c r="A16" s="1" t="n"/>
       <c r="K16" s="1" t="n"/>
-      <c r="L16" s="13" t="inlineStr">
-        <is>
-          <t>Số lượng task chưa có Spent time</t>
-        </is>
-      </c>
-      <c r="M16" s="25" t="n"/>
-      <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="n"/>
       <c r="Q16" s="1" t="n"/>
@@ -1240,17 +1233,17 @@
       <c r="X16" s="1" t="n"/>
       <c r="Y16" s="1" t="n"/>
       <c r="Z16" s="1" t="n"/>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Số lượng task chưa có Spent time</t>
+        </is>
+      </c>
+      <c r="M16" s="25" t="n"/>
+      <c r="N16" s="1" t="n"/>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="66">
       <c r="A17" s="1" t="n"/>
       <c r="K17" s="1" t="n"/>
-      <c r="L17" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task đúng hạn </t>
-        </is>
-      </c>
-      <c r="M17" s="25" t="n"/>
-      <c r="N17" s="1" t="n"/>
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="n"/>
       <c r="Q17" s="1" t="n"/>
@@ -1263,17 +1256,17 @@
       <c r="X17" s="1" t="n"/>
       <c r="Y17" s="1" t="n"/>
       <c r="Z17" s="1" t="n"/>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task đúng hạn </t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="n"/>
+      <c r="N17" s="1" t="n"/>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="66">
       <c r="A18" s="1" t="n"/>
       <c r="K18" s="1" t="n"/>
-      <c r="L18" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task trễ hạn </t>
-        </is>
-      </c>
-      <c r="M18" s="25" t="n"/>
-      <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="n"/>
       <c r="Q18" s="1" t="n"/>
@@ -1286,13 +1279,17 @@
       <c r="X18" s="1" t="n"/>
       <c r="Y18" s="1" t="n"/>
       <c r="Z18" s="1" t="n"/>
+      <c r="L18" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task trễ hạn </t>
+        </is>
+      </c>
+      <c r="M18" s="25" t="n"/>
+      <c r="N18" s="1" t="n"/>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="66">
       <c r="A19" s="1" t="n"/>
       <c r="K19" s="1" t="n"/>
-      <c r="L19" s="25" t="n"/>
-      <c r="M19" s="25" t="n"/>
-      <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="n"/>
       <c r="Q19" s="1" t="n"/>
@@ -1305,17 +1302,17 @@
       <c r="X19" s="1" t="n"/>
       <c r="Y19" s="1" t="n"/>
       <c r="Z19" s="1" t="n"/>
+      <c r="L19" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task không bị reopen </t>
+        </is>
+      </c>
+      <c r="M19" s="25" t="n"/>
+      <c r="N19" s="1" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="66">
       <c r="A20" s="1" t="n"/>
       <c r="K20" s="1" t="n"/>
-      <c r="L20" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task không bị reopen </t>
-        </is>
-      </c>
-      <c r="M20" s="25" t="n"/>
-      <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
       <c r="Q20" s="1" t="n"/>
@@ -1328,17 +1325,17 @@
       <c r="X20" s="1" t="n"/>
       <c r="Y20" s="1" t="n"/>
       <c r="Z20" s="1" t="n"/>
+      <c r="L20" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task có bị reopen </t>
+        </is>
+      </c>
+      <c r="M20" s="25" t="n"/>
+      <c r="N20" s="1" t="n"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="66">
       <c r="A21" s="1" t="n"/>
       <c r="K21" s="1" t="n"/>
-      <c r="L21" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task có bị reopen </t>
-        </is>
-      </c>
-      <c r="M21" s="25" t="n"/>
-      <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="n"/>
       <c r="Q21" s="1" t="n"/>
@@ -1355,9 +1352,6 @@
     <row r="22" ht="15.75" customHeight="1" s="66">
       <c r="A22" s="1" t="n"/>
       <c r="K22" s="1" t="n"/>
-      <c r="L22" s="1" t="n"/>
-      <c r="M22" s="1" t="n"/>
-      <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="n"/>
       <c r="Q22" s="1" t="n"/>
@@ -1374,9 +1368,6 @@
     <row r="23" ht="15.75" customHeight="1" s="66">
       <c r="A23" s="1" t="n"/>
       <c r="K23" s="1" t="n"/>
-      <c r="L23" s="1" t="n"/>
-      <c r="M23" s="1" t="n"/>
-      <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
       <c r="Q23" s="1" t="n"/>
@@ -1389,17 +1380,17 @@
       <c r="X23" s="1" t="n"/>
       <c r="Y23" s="1" t="n"/>
       <c r="Z23" s="1" t="n"/>
+      <c r="L23" s="67" t="inlineStr">
+        <is>
+          <t>Tỉ lệ (%)</t>
+        </is>
+      </c>
+      <c r="M23" s="68" t="n"/>
+      <c r="N23" s="1" t="n"/>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="66">
       <c r="A24" s="1" t="n"/>
       <c r="K24" s="1" t="n"/>
-      <c r="L24" s="67" t="inlineStr">
-        <is>
-          <t>Tỉ lệ (%)</t>
-        </is>
-      </c>
-      <c r="M24" s="68" t="n"/>
-      <c r="N24" s="1" t="n"/>
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="n"/>
       <c r="Q24" s="1" t="n"/>
@@ -1412,20 +1403,20 @@
       <c r="X24" s="1" t="n"/>
       <c r="Y24" s="1" t="n"/>
       <c r="Z24" s="1" t="n"/>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Start date / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M24" s="51">
+        <f>M13/M5*100</f>
+        <v/>
+      </c>
+      <c r="N24" s="1" t="n"/>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="66">
       <c r="A25" s="1" t="n"/>
       <c r="K25" s="1" t="n"/>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Start date / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M25" s="51">
-        <f>M13/M5*100</f>
-        <v/>
-      </c>
-      <c r="N25" s="1" t="n"/>
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
       <c r="Q25" s="1" t="n"/>
@@ -1438,20 +1429,20 @@
       <c r="X25" s="1" t="n"/>
       <c r="Y25" s="1" t="n"/>
       <c r="Z25" s="1" t="n"/>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Due date / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M25" s="51">
+        <f>M14/M5*100</f>
+        <v/>
+      </c>
+      <c r="N25" s="1" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="66">
       <c r="A26" s="1" t="n"/>
       <c r="K26" s="1" t="n"/>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Due date / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M26" s="51">
-        <f>M14/M5*100</f>
-        <v/>
-      </c>
-      <c r="N26" s="1" t="n"/>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
       <c r="Q26" s="1" t="n"/>
@@ -1464,20 +1455,20 @@
       <c r="X26" s="1" t="n"/>
       <c r="Y26" s="1" t="n"/>
       <c r="Z26" s="1" t="n"/>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Estimate / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M26" s="51">
+        <f>M15/M5*100</f>
+        <v/>
+      </c>
+      <c r="N26" s="1" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="66">
       <c r="A27" s="1" t="n"/>
       <c r="K27" s="1" t="n"/>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Estimate / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M27" s="51">
-        <f>M15/M5*100</f>
-        <v/>
-      </c>
-      <c r="N27" s="1" t="n"/>
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="n"/>
       <c r="Q27" s="1" t="n"/>
@@ -1490,20 +1481,20 @@
       <c r="X27" s="1" t="n"/>
       <c r="Y27" s="1" t="n"/>
       <c r="Z27" s="1" t="n"/>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số lượng task chưa có Spent time / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M27" s="51">
+        <f>M16/M5*100</f>
+        <v/>
+      </c>
+      <c r="N27" s="1" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="66">
       <c r="A28" s="1" t="n"/>
       <c r="K28" s="1" t="n"/>
-      <c r="L28" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số lượng task chưa có Spent time / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M28" s="51">
-        <f>M16/M5*100</f>
-        <v/>
-      </c>
-      <c r="N28" s="1" t="n"/>
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="n"/>
       <c r="Q28" s="1" t="n"/>
@@ -1516,20 +1507,20 @@
       <c r="X28" s="1" t="n"/>
       <c r="Y28" s="1" t="n"/>
       <c r="Z28" s="1" t="n"/>
+      <c r="L28" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task đúng hạn / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M28" s="51">
+        <f>M17/M5*100</f>
+        <v/>
+      </c>
+      <c r="N28" s="1" t="n"/>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="66">
       <c r="A29" s="1" t="n"/>
       <c r="K29" s="1" t="n"/>
-      <c r="L29" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task đúng hạn / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M29" s="51">
-        <f>M17/M5*100</f>
-        <v/>
-      </c>
-      <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="1" t="n"/>
       <c r="Q29" s="1" t="n"/>
@@ -1542,13 +1533,20 @@
       <c r="X29" s="1" t="n"/>
       <c r="Y29" s="1" t="n"/>
       <c r="Z29" s="1" t="n"/>
+      <c r="L29" s="25" t="inlineStr">
+        <is>
+          <t>Tổng số task trễ hạn / Tổng số task</t>
+        </is>
+      </c>
+      <c r="M29" s="51">
+        <f>M18/M5*100</f>
+        <v/>
+      </c>
+      <c r="N29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n"/>
       <c r="K30" s="1" t="n"/>
-      <c r="L30" s="25" t="n"/>
-      <c r="M30" s="51" t="n"/>
-      <c r="N30" s="1" t="n"/>
       <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="n"/>
       <c r="Q30" s="1" t="n"/>
@@ -1561,20 +1559,20 @@
       <c r="X30" s="1" t="n"/>
       <c r="Y30" s="1" t="n"/>
       <c r="Z30" s="1" t="n"/>
+      <c r="L30" s="25" t="inlineStr">
+        <is>
+          <t>Tổng số task không bị reopen / Tổng số task</t>
+        </is>
+      </c>
+      <c r="M30" s="51">
+        <f>M19/M5*100</f>
+        <v/>
+      </c>
+      <c r="N30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
       <c r="K31" s="1" t="n"/>
-      <c r="L31" s="25" t="inlineStr">
-        <is>
-          <t>Tổng số task trễ hạn / Tổng số task</t>
-        </is>
-      </c>
-      <c r="M31" s="51">
-        <f>M18/M5*100</f>
-        <v/>
-      </c>
-      <c r="N31" s="1" t="n"/>
       <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="n"/>
       <c r="Q31" s="1" t="n"/>
@@ -1587,20 +1585,20 @@
       <c r="X31" s="1" t="n"/>
       <c r="Y31" s="1" t="n"/>
       <c r="Z31" s="1" t="n"/>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task có bị reopen / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M31" s="51">
+        <f>M20/M5*100</f>
+        <v/>
+      </c>
+      <c r="N31" s="1" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n"/>
       <c r="K32" s="1" t="n"/>
-      <c r="L32" s="25" t="inlineStr">
-        <is>
-          <t>Tổng số task không bị reopen / Tổng số task</t>
-        </is>
-      </c>
-      <c r="M32" s="51">
-        <f>M20/M5*100</f>
-        <v/>
-      </c>
-      <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="n"/>
       <c r="Q32" s="1" t="n"/>
@@ -1613,18 +1611,18 @@
       <c r="X32" s="1" t="n"/>
       <c r="Y32" s="1" t="n"/>
       <c r="Z32" s="1" t="n"/>
+      <c r="L32" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng số task phát sinh / Tổng số task </t>
+        </is>
+      </c>
+      <c r="M32" s="51">
+        <f>M7/M5*100</f>
+        <v/>
+      </c>
+      <c r="N32" s="1" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="66">
-      <c r="L33" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task có bị reopen / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M33" s="51">
-        <f>M21/M5*100</f>
-        <v/>
-      </c>
-      <c r="N33" s="1" t="n"/>
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="n"/>
       <c r="Q33" s="1" t="n"/>
@@ -1637,18 +1635,18 @@
       <c r="X33" s="1" t="n"/>
       <c r="Y33" s="1" t="n"/>
       <c r="Z33" s="1" t="n"/>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time / Tổng thời gian làm việc theo lịch công ty</t>
+        </is>
+      </c>
+      <c r="M33" s="51">
+        <f>M10/M8*100</f>
+        <v/>
+      </c>
+      <c r="N33" s="1" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="66">
-      <c r="L34" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng số task phát sinh / Tổng số task </t>
-        </is>
-      </c>
-      <c r="M34" s="51">
-        <f>M7/M5*100</f>
-        <v/>
-      </c>
-      <c r="N34" s="1" t="n"/>
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="n"/>
       <c r="Q34" s="1" t="n"/>
@@ -1661,11 +1659,18 @@
       <c r="X34" s="1" t="n"/>
       <c r="Y34" s="1" t="n"/>
       <c r="Z34" s="1" t="n"/>
+      <c r="L34" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tổng thời gian Spent time / Tổng thời gian Estimate </t>
+        </is>
+      </c>
+      <c r="M34" s="51">
+        <f>M10/M9*100</f>
+        <v/>
+      </c>
+      <c r="N34" s="1" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="66">
-      <c r="L35" s="25" t="n"/>
-      <c r="M35" s="51" t="n"/>
-      <c r="N35" s="1" t="n"/>
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="n"/>
       <c r="Q35" s="1" t="n"/>
@@ -1678,18 +1683,18 @@
       <c r="X35" s="1" t="n"/>
       <c r="Y35" s="1" t="n"/>
       <c r="Z35" s="1" t="n"/>
+      <c r="L35" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time của task kế hoạch / Tổng thời gian Spent time</t>
+        </is>
+      </c>
+      <c r="M35" s="51">
+        <f>M11/M10*100</f>
+        <v/>
+      </c>
+      <c r="N35" s="1" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="66">
-      <c r="L36" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time / Tổng thời gian làm việc theo lịch công ty</t>
-        </is>
-      </c>
-      <c r="M36" s="51">
-        <f>M10/M8*100</f>
-        <v/>
-      </c>
-      <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="n"/>
       <c r="Q36" s="1" t="n"/>
@@ -1702,18 +1707,18 @@
       <c r="X36" s="1" t="n"/>
       <c r="Y36" s="1" t="n"/>
       <c r="Z36" s="1" t="n"/>
+      <c r="L36" s="25" t="inlineStr">
+        <is>
+          <t>Tổng thời gian Spent time của task phát sinh / Tổng thời gian Spent time</t>
+        </is>
+      </c>
+      <c r="M36" s="51">
+        <f>M12/M10*100</f>
+        <v/>
+      </c>
+      <c r="N36" s="1" t="n"/>
     </row>
     <row r="37">
-      <c r="L37" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tổng thời gian Spent time / Tổng thời gian Estimate </t>
-        </is>
-      </c>
-      <c r="M37" s="51">
-        <f>M10/M9*100</f>
-        <v/>
-      </c>
-      <c r="N37" s="1" t="n"/>
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="n"/>
       <c r="Q37" s="1" t="n"/>
@@ -1728,16 +1733,6 @@
       <c r="Z37" s="1" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="66">
-      <c r="L38" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time của task kế hoạch / Tổng thời gian Spent time</t>
-        </is>
-      </c>
-      <c r="M38" s="51">
-        <f>M11/M10*100</f>
-        <v/>
-      </c>
-      <c r="N38" s="1" t="n"/>
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="n"/>
       <c r="Q38" s="1" t="n"/>
@@ -1752,16 +1747,6 @@
       <c r="Z38" s="1" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="66">
-      <c r="L39" s="25" t="inlineStr">
-        <is>
-          <t>Tổng thời gian Spent time của task phát sinh / Tổng thời gian Spent time</t>
-        </is>
-      </c>
-      <c r="M39" s="51">
-        <f>M12/M10*100</f>
-        <v/>
-      </c>
-      <c r="N39" s="1" t="n"/>
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="n"/>
       <c r="Q39" s="1" t="n"/>
@@ -2748,7 +2733,7 @@
     <row r="1010" ht="15.75" customHeight="1" s="66"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L23:M23"/>
     <mergeCell ref="L4:M4"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
@@ -3074,7 +3059,7 @@
         <v>0.25</v>
       </c>
       <c r="F15" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M27/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M26/100)</f>
         <v/>
       </c>
       <c r="G15" s="75">
@@ -3182,7 +3167,7 @@
         <v>0.25</v>
       </c>
       <c r="F20" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M25/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M24/100)</f>
         <v/>
       </c>
       <c r="G20" s="75">
@@ -3290,7 +3275,7 @@
         <v>0.25</v>
       </c>
       <c r="F25" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M26/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M25/100)</f>
         <v/>
       </c>
       <c r="G25" s="75">
@@ -3398,7 +3383,7 @@
         <v>0.25</v>
       </c>
       <c r="F30" s="76">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M28/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M27/100)</f>
         <v/>
       </c>
       <c r="G30" s="75">
@@ -3510,7 +3495,7 @@
         <v>3</v>
       </c>
       <c r="F35" s="75">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M36)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M33)</f>
         <v/>
       </c>
       <c r="G35" s="75">
@@ -3622,7 +3607,7 @@
         <v>3</v>
       </c>
       <c r="F40" s="83">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M31/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M29/100)</f>
         <v/>
       </c>
       <c r="G40" s="81">
@@ -3730,7 +3715,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="83">
-        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M33/100)</f>
+        <f>IF('Báo cáo công việc'!M5=0,"",'Báo cáo công việc'!M31/100)</f>
         <v/>
       </c>
       <c r="G45" s="81">

</xml_diff>